<commit_message>
Remanning the timestamp 00:00:00 issue
</commit_message>
<xml_diff>
--- a/test_data/data_merge_testdata_1.xlsx
+++ b/test_data/data_merge_testdata_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git clone projects\Data-Merge-Utility-DMU-\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FAE01E2-6702-4C60-803F-423FE8B4307C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36F3E151-5B25-41A3-8E07-C45889E6CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>日期</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -51,15 +51,8 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Junior</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>负责人1</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>负责人2</t>
   </si>
   <si>
     <t>一级</t>
@@ -392,7 +385,7 @@
   <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" customWidth="1"/>
     <col min="3" max="3" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -424,28 +417,14 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1">
-        <v>45813</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
-      </c>
+      <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>

</xml_diff>